<commit_message>
Add event and assessment support to validation spreadsheets
Add start and end time to log
Improve methods for pulling event information out of log files
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/Dehydration/Dehydration.xlsx
+++ b/data/human/adult/validation/Scenarios/Dehydration/Dehydration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\Scenarios\Dehydration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E069171D-74E8-478E-8587-79264869D0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697F28AE-6633-4998-8F43-5D3E1ACD6ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="17250" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23700" windowHeight="15795" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="10" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="117">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -299,18 +299,12 @@
     <t>{v} &gt; {Mild:1}</t>
   </si>
   <si>
-    <t xml:space="preserve"> {v} = "Dark Yellow"</t>
-  </si>
-  <si>
     <t>{v} = {Mild:1}</t>
   </si>
   <si>
     <t>{v} &lt;= {Mild:1}</t>
   </si>
   <si>
-    <t>{v} = "Dark Yellow" or {v} = "Brown"</t>
-  </si>
-  <si>
     <t>{v} &lt; {Healthy}</t>
   </si>
   <si>
@@ -347,16 +341,52 @@
     <t>Assessment</t>
   </si>
   <si>
-    <t>Urinalysis::UrineColor</t>
-  </si>
-  <si>
     <t>Healthy Dehydration</t>
   </si>
   <si>
-    <t>Baseline patient dehydration scenarios.</t>
-  </si>
-  <si>
     <t>Increase and &lt;100 bpm</t>
+  </si>
+  <si>
+    <t>Event</t>
+  </si>
+  <si>
+    <t>MildDehydration-ActiveFraction</t>
+  </si>
+  <si>
+    <t>MildDehydration-FinalState</t>
+  </si>
+  <si>
+    <t>{v} = 1.0</t>
+  </si>
+  <si>
+    <t>{v} = True</t>
+  </si>
+  <si>
+    <t>SevereDehydration-ActiveFraction</t>
+  </si>
+  <si>
+    <t>SevereDehydration-FinalState</t>
+  </si>
+  <si>
+    <t>ModerateDehydration-ActiveFraction</t>
+  </si>
+  <si>
+    <t>ModerateDehydration-FinalState</t>
+  </si>
+  <si>
+    <t>Good=2, Fair=5</t>
+  </si>
+  <si>
+    <t>Baseline patient dehydration scenario.</t>
+  </si>
+  <si>
+    <t>Urinalysis-Color</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> {v} = "DarkYellow"</t>
+  </si>
+  <si>
+    <t>{v} = "DarkYellow" or {v} = "Brown"</t>
   </si>
 </sst>
 </file>
@@ -569,7 +599,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -628,6 +658,9 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1095,49 +1128,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="29"/>
       <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A2" s="41" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="41"/>
+      <c r="A2" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="42"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="41" t="s">
-        <v>105</v>
-      </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="E2" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
     </row>
     <row r="3" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
       <c r="F3" s="16"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
@@ -1150,11 +1183,11 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="26"/>
       <c r="G4" s="4"/>
       <c r="H4" s="15"/>
     </row>
@@ -1168,62 +1201,62 @@
       <c r="C5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="27"/>
+      <c r="E5" s="28"/>
       <c r="F5" s="16"/>
-      <c r="G5" s="28" t="s">
+      <c r="G5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="28"/>
+      <c r="H5" s="29"/>
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="30"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="32"/>
     </row>
     <row r="7" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="39"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36"/>
     </row>
     <row r="9" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
       <c r="F9" s="17"/>
       <c r="G9" s="1" t="s">
         <v>7</v>
@@ -1236,13 +1269,13 @@
       <c r="A10" s="12">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="26"/>
       <c r="G10" s="13"/>
       <c r="H10" s="15"/>
     </row>
@@ -1250,13 +1283,13 @@
       <c r="A11" s="10">
         <v>1</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="26"/>
       <c r="G11" s="4"/>
       <c r="H11" s="15" t="s">
         <v>25</v>
@@ -1273,7 +1306,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>15</v>
@@ -1438,7 +1471,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AMJ23"/>
+  <dimension ref="A1:AMJ25"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="8" customWidth="1"/>
@@ -1446,56 +1479,56 @@
     <col min="3" max="3" width="21.28515625" style="8" customWidth="1"/>
     <col min="4" max="4" width="33.28515625" style="8" customWidth="1"/>
     <col min="5" max="5" width="39" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="30.5703125" style="8" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="37.28515625" style="9" customWidth="1"/>
     <col min="9" max="1024" width="11.5703125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="29"/>
       <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="41"/>
+      <c r="B2" s="42"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
     </row>
     <row r="3" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
       <c r="F3" s="16"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
@@ -1508,13 +1541,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="26"/>
       <c r="G4" s="4"/>
       <c r="H4" s="15"/>
     </row>
@@ -1528,62 +1561,62 @@
       <c r="C5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="27"/>
+      <c r="E5" s="28"/>
       <c r="F5" s="16"/>
-      <c r="G5" s="28" t="s">
+      <c r="G5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="28"/>
+      <c r="H5" s="29"/>
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="30"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="32"/>
     </row>
     <row r="7" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="39"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36"/>
     </row>
     <row r="9" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
       <c r="F9" s="17"/>
       <c r="G9" s="1" t="s">
         <v>7</v>
@@ -1596,13 +1629,13 @@
       <c r="A10" s="12">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="26"/>
       <c r="G10" s="13"/>
       <c r="H10" s="15"/>
     </row>
@@ -1610,13 +1643,13 @@
       <c r="A11" s="10">
         <v>1</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="26"/>
       <c r="G11" s="4"/>
       <c r="H11" s="15" t="s">
         <v>25</v>
@@ -1633,7 +1666,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>15</v>
@@ -1659,7 +1692,7 @@
         <v>64</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>52</v>
@@ -1681,7 +1714,7 @@
         <v>34</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>53</v>
@@ -1704,14 +1737,14 @@
         <v>18</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>67</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H15" s="2"/>
       <c r="AMJ15"/>
@@ -1727,7 +1760,7 @@
         <v>36</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>52</v>
@@ -1750,7 +1783,7 @@
         <v>37</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>54</v>
@@ -1773,7 +1806,7 @@
         <v>36</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>53</v>
@@ -1796,7 +1829,7 @@
         <v>35</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>53</v>
@@ -1842,7 +1875,7 @@
         <v>39</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>53</v>
@@ -1879,16 +1912,16 @@
     </row>
     <row r="23" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>81</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>59</v>
@@ -1901,6 +1934,40 @@
         <v>61</v>
       </c>
       <c r="AMJ23"/>
+    </row>
+    <row r="24" spans="1:1024" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" t="s">
+        <v>112</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="21"/>
+    </row>
+    <row r="25" spans="1:1024" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -1931,7 +1998,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70C22A4B-7DC3-4468-B3AD-DF3C2884C93E}">
-  <dimension ref="A1:AMJ25"/>
+  <dimension ref="A1:AMJ27"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="8" customWidth="1"/>
@@ -1939,57 +2006,57 @@
     <col min="3" max="3" width="21.28515625" style="8" customWidth="1"/>
     <col min="4" max="4" width="35.5703125" style="8" customWidth="1"/>
     <col min="5" max="5" width="39" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.42578125" style="8" customWidth="1"/>
     <col min="8" max="8" width="35.85546875" style="9" bestFit="1" customWidth="1"/>
     <col min="9" max="1024" width="11.5703125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="29"/>
       <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="41"/>
+      <c r="B2" s="42"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="43"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -2001,13 +2068,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="26"/>
       <c r="G4" s="4"/>
       <c r="H4" s="15"/>
     </row>
@@ -2021,63 +2088,63 @@
       <c r="C5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="27"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="28" t="s">
+      <c r="E5" s="28"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="28"/>
+      <c r="H5" s="29"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
-      <c r="D6" s="36" t="s">
+      <c r="D6" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="31"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="32"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="36" t="s">
+      <c r="D8" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="37"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36"/>
     </row>
     <row r="9" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="42"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="43"/>
       <c r="G9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2089,13 +2156,13 @@
       <c r="A10" s="12">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="26"/>
       <c r="G10" s="13"/>
       <c r="H10" s="15"/>
     </row>
@@ -2103,13 +2170,13 @@
       <c r="A11" s="10">
         <v>1</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="26"/>
       <c r="G11" s="4"/>
       <c r="H11" s="15" t="s">
         <v>25</v>
@@ -2126,7 +2193,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>15</v>
@@ -2262,7 +2329,7 @@
         <v>36</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>52</v>
@@ -2284,7 +2351,7 @@
         <v>37</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>54</v>
@@ -2407,16 +2474,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>81</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>59</v>
@@ -2426,6 +2493,40 @@
         <v>71</v>
       </c>
       <c r="H25" s="2"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="21"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -2456,7 +2557,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B282E4DC-0B8D-487E-A497-DD64F028D134}">
-  <dimension ref="A1:AMJ26"/>
+  <dimension ref="A1:AMJ28"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="8" customWidth="1"/>
@@ -2464,57 +2565,57 @@
     <col min="3" max="3" width="21.28515625" style="8" customWidth="1"/>
     <col min="4" max="4" width="35.5703125" style="8" customWidth="1"/>
     <col min="5" max="5" width="61.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.5703125" style="8" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="33.85546875" style="9" customWidth="1"/>
     <col min="9" max="1024" width="11.5703125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="29"/>
       <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="41"/>
+      <c r="B2" s="42"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="43"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -2526,13 +2627,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="26"/>
       <c r="G4" s="4"/>
       <c r="H4" s="15"/>
     </row>
@@ -2546,63 +2647,63 @@
       <c r="C5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="27"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="28" t="s">
+      <c r="E5" s="28"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="28"/>
+      <c r="H5" s="29"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
-      <c r="D6" s="36" t="s">
+      <c r="D6" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="31"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="32"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="36" t="s">
+      <c r="D8" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="37"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36"/>
     </row>
     <row r="9" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="42"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="43"/>
       <c r="G9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2614,13 +2715,13 @@
       <c r="A10" s="12">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="26"/>
       <c r="G10" s="13"/>
       <c r="H10" s="15"/>
     </row>
@@ -2628,13 +2729,13 @@
       <c r="A11" s="10">
         <v>1</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="26"/>
       <c r="G11" s="4"/>
       <c r="H11" s="15" t="s">
         <v>25</v>
@@ -2651,7 +2752,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>15</v>
@@ -2677,7 +2778,7 @@
         <v>64</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>52</v>
@@ -2699,7 +2800,7 @@
         <v>34</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>53</v>
@@ -2721,7 +2822,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>74</v>
@@ -2743,7 +2844,7 @@
         <v>18</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>76</v>
@@ -2765,7 +2866,7 @@
         <v>35</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>77</v>
@@ -2787,7 +2888,7 @@
         <v>36</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>52</v>
@@ -2809,7 +2910,7 @@
         <v>36</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>59</v>
@@ -2832,7 +2933,7 @@
         <v>37</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -2854,7 +2955,7 @@
         <v>36</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>53</v>
@@ -2876,7 +2977,7 @@
         <v>35</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>53</v>
@@ -2898,7 +2999,7 @@
         <v>38</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>53</v>
@@ -2920,7 +3021,7 @@
         <v>39</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>67</v>
@@ -2942,7 +3043,7 @@
         <v>40</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>53</v>
@@ -2955,16 +3056,16 @@
     </row>
     <row r="26" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>81</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>76</v>
@@ -2974,6 +3075,40 @@
         <v>80</v>
       </c>
       <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="1:1024" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" t="s">
+        <v>112</v>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="H27" s="21"/>
+    </row>
+    <row r="28" spans="1:1024" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -2994,7 +3129,7 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>